<commit_message>
New Pet: orientações de preenchimento dos diferenciais
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016M21DdQvw1tBZmQFRKKNVQ
</commit_message>
<xml_diff>
--- a/dados_raw/new_pet/novos/Pedido_informacoes_Grupo_New_Pet.xlsx
+++ b/dados_raw/new_pet/novos/Pedido_informacoes_Grupo_New_Pet.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +27,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00C00000"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -54,27 +63,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
+        <fgColor rgb="FFC00000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00548235"/>
+        <fgColor rgb="FF548235"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,23 +97,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </left>
       <right style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </right>
       <top style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BBBBBB"/>
+        <color rgb="FFBBBBBB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -140,9 +150,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -214,6 +227,49 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Grupo Start</author>
+  </authors>
+  <commentList>
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t>Escreva 1 frase com a composição que mais diferencia o produto, com números do rótulo.
+Formato: [ingrediente/nutriente] + [quantidade].
+Exemplo do formato (troque pelos dados reais): 'Proteína bruta mínima de XX% com [fonte de proteína]'.</t>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0" shapeId="0">
+      <text>
+        <t>Escreva 1 frase com o benefício e o ingrediente/nutriente que o causa. Só o que a marca pode comprovar.
+Formato: [benefício] graças a [ingrediente/nutriente].
+Exemplo do formato: 'Ajuda na saúde da pelagem com [nutriente]'.</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
+      <text>
+        <t>Escreva 1 frase dizendo para qual animal o produto é indicado e por quê.
+Formato: indicado para [espécie + fase + porte] com [característica do grão/nutrição adequada].
+Exemplo do formato: 'Indicado para cães adultos de raças pequenas, com grãos de tamanho adequado'.</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
+      <text>
+        <t>Só preencha se for verdade e constar no rótulo/documentos da marca.
+Exemplo do formato: 'Sem corantes artificiais'.</t>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="0" shapeId="0">
+      <text>
+        <t>Escreva algo concreto e útil ao cliente: rendimento em dias para um animal de tamanho X, tipo de embalagem, selo da marca etc.
+Exemplo do formato: 'Pacote de X kg rende cerca de X dias para um cão de X kg'.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -505,13 +561,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Grupo New Pet — informações complementares para cadastro na Amazon</t>
@@ -519,7 +575,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -528,7 +584,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Faltam as informações da aba 'Produtos'. Preencha as células AMARELAS. A linha acima do título de cada coluna indica se é OBRIGATÓRIO (vermelho) ou OPCIONAL (verde).</t>
@@ -542,7 +598,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>• Aba 'Confirmar': pontos em que os dados enviados estão errados ou inconsistentes. Precisamos da resposta correta. O item 1 (EAN repetido) impede o cadastro se não for corrigido.</t>
@@ -567,6 +623,62 @@
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>• Imagens serão tratadas em outra etapa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>COMO PREENCHER OS DIFERENCIAIS (viram os tópicos do anúncio na Amazon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>• Cada diferencial é 1 frase curta (até cerca de 200 caracteres), uma ideia por coluna, sem repetir o nome do produto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>• Ordem sugerida: 1) Nutrição/composição, 2) Benefício à saúde, 3) Indicação (para quem é), 4) Qualidade/ausência de ingredientes, 5) Embalagem/rendimento/marca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>• Use números sempre que existirem (%, kg, dias de rendimento). Prefira dados do rótulo e dos documentos da marca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>• Escreva só o que a marca pode comprovar. Não inventar benefícios, não citar cura ou tratamento de doenças.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>• NÃO usar: preço, 'econômico', 'barato', 'oferta', 'promoção', 'frete grátis', 'melhor do mercado', 'o melhor', 'nº 1'. A Amazon bloqueia esses termos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>• Os exemplos nos comentários das colunas mostram só o FORMATO da frase; troque pelos dados reais de cada produto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Produtos da mesma linha podem ter diferenciais parecidos, mas ajuste o que muda (fase de vida, porte, tamanho do pacote, rendimento).</t>
         </is>
       </c>
     </row>
@@ -581,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK18"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -597,38 +709,23 @@
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="38" customWidth="1" min="14" max="14"/>
-    <col width="38" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="38" customWidth="1" min="17" max="17"/>
-    <col width="38" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" min="14" max="18"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
+    <col width="44" customWidth="1" min="18" max="18"/>
     <col width="50" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
-    <col width="28" customWidth="1" min="22" max="22"/>
+    <col width="28" customWidth="1" min="20" max="22"/>
     <col width="24" customWidth="1" min="23" max="23"/>
     <col width="42" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
     <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
-    <col width="11" customWidth="1" min="34" max="34"/>
-    <col width="11" customWidth="1" min="35" max="35"/>
-    <col width="11" customWidth="1" min="36" max="36"/>
-    <col width="20" customWidth="1" min="37" max="37"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
       <c r="F1" s="3" t="inlineStr">
         <is>
           <t>OBRIGATÓRIO</t>
@@ -734,9 +831,9 @@
           <t>OBRIGATÓRIO</t>
         </is>
       </c>
-      <c r="AA1" s="4" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>OBRIGATÓRIO</t>
         </is>
       </c>
       <c r="AB1" s="3" t="inlineStr">
@@ -749,48 +846,8 @@
           <t>OBRIGATÓRIO</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AE1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AF1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AG1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AH1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AI1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AJ1" s="3" t="inlineStr">
-        <is>
-          <t>OBRIGATÓRIO</t>
-        </is>
-      </c>
-      <c r="AK1" s="4" t="inlineStr">
-        <is>
-          <t>OPCIONAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="90" customHeight="1">
+    </row>
+    <row r="2" ht="140" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>SKU</t>
@@ -858,27 +915,32 @@
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>Diferencial 1</t>
+          <t>Diferencial 1 — NUTRIÇÃO: o que tem de mais importante na composição
+(ex.: fonte principal de proteína, % mínima de proteína, nutrientes que o rótulo destaca)</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Diferencial 2</t>
+          <t>Diferencial 2 — BENEFÍCIO para o animal: o que o produto faz pela saúde
+(ex.: pelagem, digestão, ossos e articulações, imunidade)</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Diferencial 3</t>
+          <t>Diferencial 3 — INDICAÇÃO: para quem é e como usar
+(ex.: fase de vida, porte da raça, necessidades especiais)</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>Diferencial 4</t>
+          <t>Diferencial 4 (opcional) — QUALIDADE: o que NÃO leva ou selos
+(ex.: sem corantes artificiais, sem transgênicos, certificações)</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>Diferencial 5</t>
+          <t>Diferencial 5 (opcional) — EMBALAGEM / RENDIMENTO / MARCA
+(ex.: pacote com fecho, rendimento diário, tradição da marca)</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -923,57 +985,17 @@
       </c>
       <c r="AA2" s="5" t="inlineStr">
         <is>
-          <t>Cor predominante do produto/embalagem</t>
+          <t>Registro no MAPA / certificação (número, ou 'Não aplicável')</t>
         </is>
       </c>
       <c r="AB2" s="5" t="inlineStr">
         <is>
-          <t>Registro no MAPA / certificação (número, ou 'Não aplicável')</t>
+          <t>Fabricante real (razão social)</t>
         </is>
       </c>
       <c r="AC2" s="5" t="inlineStr">
         <is>
-          <t>Fabricante real (razão social)</t>
-        </is>
-      </c>
-      <c r="AD2" s="5" t="inlineStr">
-        <is>
           <t>Preço sugerido PDV (R$)</t>
-        </is>
-      </c>
-      <c r="AE2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: peso (kg)</t>
-        </is>
-      </c>
-      <c r="AF2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: comprimento (cm)</t>
-        </is>
-      </c>
-      <c r="AG2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: largura (cm)</t>
-        </is>
-      </c>
-      <c r="AH2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: altura (cm)</t>
-        </is>
-      </c>
-      <c r="AI2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: camadas por palete</t>
-        </is>
-      </c>
-      <c r="AJ2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: caixas por camada</t>
-        </is>
-      </c>
-      <c r="AK2" s="5" t="inlineStr">
-        <is>
-          <t>Caixa master: código de barras da caixa (DUN-14/GTIN), se existir</t>
         </is>
       </c>
     </row>
@@ -1025,42 +1047,6 @@
       <c r="AA3" s="8" t="n"/>
       <c r="AB3" s="8" t="n"/>
       <c r="AC3" s="8" t="n"/>
-      <c r="AD3" s="8" t="n"/>
-      <c r="AE3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK3" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -1110,42 +1096,6 @@
       <c r="AA4" s="8" t="n"/>
       <c r="AB4" s="8" t="n"/>
       <c r="AC4" s="8" t="n"/>
-      <c r="AD4" s="8" t="n"/>
-      <c r="AE4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK4" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1195,42 +1145,6 @@
       <c r="AA5" s="8" t="n"/>
       <c r="AB5" s="8" t="n"/>
       <c r="AC5" s="8" t="n"/>
-      <c r="AD5" s="8" t="n"/>
-      <c r="AE5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK5" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1280,42 +1194,6 @@
       <c r="AA6" s="8" t="n"/>
       <c r="AB6" s="8" t="n"/>
       <c r="AC6" s="8" t="n"/>
-      <c r="AD6" s="8" t="n"/>
-      <c r="AE6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK6" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -1365,42 +1243,6 @@
       <c r="AA7" s="8" t="n"/>
       <c r="AB7" s="8" t="n"/>
       <c r="AC7" s="8" t="n"/>
-      <c r="AD7" s="8" t="n"/>
-      <c r="AE7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK7" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -1450,14 +1292,6 @@
       <c r="AA8" s="8" t="n"/>
       <c r="AB8" s="8" t="n"/>
       <c r="AC8" s="8" t="n"/>
-      <c r="AD8" s="8" t="n"/>
-      <c r="AE8" s="8" t="n"/>
-      <c r="AF8" s="8" t="n"/>
-      <c r="AG8" s="8" t="n"/>
-      <c r="AH8" s="8" t="n"/>
-      <c r="AI8" s="8" t="n"/>
-      <c r="AJ8" s="8" t="n"/>
-      <c r="AK8" s="8" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1507,42 +1341,6 @@
       <c r="AA9" s="8" t="n"/>
       <c r="AB9" s="8" t="n"/>
       <c r="AC9" s="8" t="n"/>
-      <c r="AD9" s="8" t="n"/>
-      <c r="AE9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK9" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1592,42 +1390,6 @@
       <c r="AA10" s="8" t="n"/>
       <c r="AB10" s="8" t="n"/>
       <c r="AC10" s="8" t="n"/>
-      <c r="AD10" s="8" t="n"/>
-      <c r="AE10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK10" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1677,14 +1439,6 @@
       <c r="AA11" s="8" t="n"/>
       <c r="AB11" s="8" t="n"/>
       <c r="AC11" s="8" t="n"/>
-      <c r="AD11" s="8" t="n"/>
-      <c r="AE11" s="8" t="n"/>
-      <c r="AF11" s="8" t="n"/>
-      <c r="AG11" s="8" t="n"/>
-      <c r="AH11" s="8" t="n"/>
-      <c r="AI11" s="8" t="n"/>
-      <c r="AJ11" s="8" t="n"/>
-      <c r="AK11" s="8" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1734,42 +1488,6 @@
       <c r="AA12" s="8" t="n"/>
       <c r="AB12" s="8" t="n"/>
       <c r="AC12" s="8" t="n"/>
-      <c r="AD12" s="8" t="n"/>
-      <c r="AE12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK12" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1819,14 +1537,6 @@
       <c r="AA13" s="8" t="n"/>
       <c r="AB13" s="8" t="n"/>
       <c r="AC13" s="8" t="n"/>
-      <c r="AD13" s="8" t="n"/>
-      <c r="AE13" s="8" t="n"/>
-      <c r="AF13" s="8" t="n"/>
-      <c r="AG13" s="8" t="n"/>
-      <c r="AH13" s="8" t="n"/>
-      <c r="AI13" s="8" t="n"/>
-      <c r="AJ13" s="8" t="n"/>
-      <c r="AK13" s="8" t="n"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -1876,14 +1586,6 @@
       <c r="AA14" s="8" t="n"/>
       <c r="AB14" s="8" t="n"/>
       <c r="AC14" s="8" t="n"/>
-      <c r="AD14" s="8" t="n"/>
-      <c r="AE14" s="8" t="n"/>
-      <c r="AF14" s="8" t="n"/>
-      <c r="AG14" s="8" t="n"/>
-      <c r="AH14" s="8" t="n"/>
-      <c r="AI14" s="8" t="n"/>
-      <c r="AJ14" s="8" t="n"/>
-      <c r="AK14" s="8" t="n"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -1933,42 +1635,6 @@
       <c r="AA15" s="8" t="n"/>
       <c r="AB15" s="8" t="n"/>
       <c r="AC15" s="8" t="n"/>
-      <c r="AD15" s="8" t="n"/>
-      <c r="AE15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK15" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -2018,14 +1684,6 @@
       <c r="AA16" s="8" t="n"/>
       <c r="AB16" s="8" t="n"/>
       <c r="AC16" s="8" t="n"/>
-      <c r="AD16" s="8" t="n"/>
-      <c r="AE16" s="8" t="n"/>
-      <c r="AF16" s="8" t="n"/>
-      <c r="AG16" s="8" t="n"/>
-      <c r="AH16" s="8" t="n"/>
-      <c r="AI16" s="8" t="n"/>
-      <c r="AJ16" s="8" t="n"/>
-      <c r="AK16" s="8" t="n"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -2075,14 +1733,6 @@
       <c r="AA17" s="8" t="n"/>
       <c r="AB17" s="8" t="n"/>
       <c r="AC17" s="8" t="n"/>
-      <c r="AD17" s="8" t="n"/>
-      <c r="AE17" s="8" t="n"/>
-      <c r="AF17" s="8" t="n"/>
-      <c r="AG17" s="8" t="n"/>
-      <c r="AH17" s="8" t="n"/>
-      <c r="AI17" s="8" t="n"/>
-      <c r="AJ17" s="8" t="n"/>
-      <c r="AK17" s="8" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -2132,42 +1782,6 @@
       <c r="AA18" s="8" t="n"/>
       <c r="AB18" s="8" t="n"/>
       <c r="AC18" s="8" t="n"/>
-      <c r="AD18" s="8" t="n"/>
-      <c r="AE18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AF18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AG18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AH18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AI18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AJ18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AK18" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2179,6 +1793,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2213,7 +1828,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>1192 e 1221</t>
@@ -2224,9 +1839,9 @@
           <t>EAN REPETIDO: os SKUs 1192 (Buzz Cat Adultos Mix 1 kg) e 1221 (Buzz Cat Adultos Mix 2,5 kg) estão com o mesmo EAN 7898968541078. Cada tamanho precisa ter EAN próprio e a Amazon não aceita dois produtos com o mesmo código. Qual é o EAN correto de cada um?</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="C2" s="11" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>1148, 1916, 1147, 1149, 1900</t>
@@ -2237,7 +1852,7 @@
           <t>A marca aparece como 'Natural Dots' nos SKUs 1148 e 1916 e como 'New Dots' nos 1147, 1149 e 1900. São marcas/linhas diferentes? Qual é o nome exato da marca de cada produto?</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr"/>
+      <c r="C3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -2250,7 +1865,7 @@
           <t>As rações 'Buzz Cat' (gatos) estão com a marca 'Buzz Dog'. A marca correta é 'Buzz Cat' ou 'Buzz Dog'?</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr"/>
+      <c r="C4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -2263,7 +1878,7 @@
           <t>O campo Fabricante está em branco. Qual é o fabricante (razão social)?</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr"/>
+      <c r="C5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -2276,9 +1891,9 @@
           <t>O nome diz 'Cães Adultos', mas a descrição enviada diz 'Cães Filhotes'. Qual está certo?</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="C6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>1916</t>
@@ -2289,9 +1904,9 @@
           <t>O nome diz 'Cães Adultos Todas as Raças', mas a descrição enviada diz 'Premium Especial Cães Raças Pequenas'. Qual está certo? Confirmar também o EAN 7898968541276 (começa igual aos da linha Buzz Dog).</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="C7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -2302,9 +1917,9 @@
           <t>O campo 'Tamanho' enviado é inconsistente (ex.: 1147/1148/1149/1900/1916/1279 'Grande'; 1184, 1186, 1189 e 1192 'Pequeno'; 1187, 1190, 1221 e 1193 'Medio'/'Médio'). Esse campo se refere ao tamanho da embalagem, ao porte do animal ou a outra coisa? Qual o valor correto de cada produto?</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="C8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -2315,7 +1930,7 @@
           <t>O sabor está como 'carne' em todos (inclusive ração de gato). É só 'carne' mesmo ou há outros sabores/ingredientes principais? Informe o sabor exato na aba Produtos.</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr"/>
+      <c r="C9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -2328,9 +1943,9 @@
           <t>Validade de 540 dias; nos demais é 365 dias. Confirmar o prazo correto de cada um.</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="C10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>1184, 1186, 1189, 1192 (12 un.) e 1220, 1221 (6 un.)</t>
@@ -2341,7 +1956,7 @@
           <t>A quantidade por caixa master é 12 (1 kg) e 6 (2,5 kg). As medidas enviadas (ex.: 8 × 18 × 34 cm) são da embalagem unitária ou da caixa? Precisamos também das medidas e peso da caixa master (colunas da aba Produtos).</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr"/>
+      <c r="C11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -2354,9 +1969,9 @@
           <t>O peso enviado (ex.: 10,1 kg) é o peso do produto ou o peso bruto com a embalagem?</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13">
+      <c r="C12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -2367,9 +1982,9 @@
           <t>A 'descrição' enviada é igual ao nome do produto. Precisamos de um texto de descrição de verdade (coluna na aba Produtos).</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14">
+      <c r="C13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -2380,7 +1995,7 @@
           <t>Confirmar o NCM 23.09.90.10 para todos (inclusive ração para gatos) e o fabricante real, pois foi enviado 'Grupo New Pet'.</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr"/>
+      <c r="C14" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
New Pet: orientação da descrição comercial
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016M21DdQvw1tBZmQFRKKNVQ
</commit_message>
<xml_diff>
--- a/dados_raw/new_pet/novos/Pedido_informacoes_Grupo_New_Pet.xlsx
+++ b/dados_raw/new_pet/novos/Pedido_informacoes_Grupo_New_Pet.xlsx
@@ -266,6 +266,18 @@
       <text>
         <t>Escreva algo concreto e útil ao cliente: rendimento em dias para um animal de tamanho X, tipo de embalagem, selo da marca etc.
 Exemplo do formato: 'Pacote de X kg rende cerca de X dias para um cão de X kg'.</t>
+      </text>
+    </comment>
+    <comment ref="S2" authorId="0" shapeId="0">
+      <text>
+        <t>A descrição é o texto que o cliente lê para decidir a compra. Escrever o nome do produto aqui NÃO é aceito: precisamos de um texto de verdade.
+Estrutura sugerida (1 a 2 frases em cada):
+1) Para quem é: espécie, fase de vida, porte.
+2) O que tem de especial: ingredientes, nutrientes, processo de fabricação.
+3) O que faz pelo animal: pelagem, digestão, energia etc. (só o que a marca comprova).
+4) Como usar/dar: referência à tabela de alimentação e transição de ração.
+Formato do texto (troque pelos dados reais): 'A [linha/marca] é uma ração [fase] para [espécie] de porte [porte], feita com [ingredientes principais]. Contém [nutriente] que ajuda [benefício]. Siga a tabela de alimentação da embalagem e faça a transição gradual com a ração anterior.'
+Não usar: preço, 'oferta', 'promoção', 'frete grátis', 'o melhor', cura/tratamento de doenças. Não copiar os diferenciais palavra por palavra.</t>
       </text>
     </comment>
   </commentList>
@@ -561,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -679,6 +691,41 @@
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>• Produtos da mesma linha podem ter diferenciais parecidos, mas ajuste o que muda (fase de vida, porte, tamanho do pacote, rendimento).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>COMO PREENCHER A DESCRIÇÃO COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• NÃO colocar o nome do produto: ele já aparece no título do anúncio. Precisamos de um texto corrido, de 3 a 5 frases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>• Conteúdo: 1) para quem é (espécie, fase, porte); 2) o que tem de especial (ingredientes, nutrientes); 3) o que faz pelo animal; 4) como usar (tabela de alimentação, transição de ração).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>• Não repetir os diferenciais palavra por palavra; a descrição complementa os tópicos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>• Mesmas regras dos diferenciais: sem preço, 'oferta', 'promoção', 'frete grátis', 'o melhor' e sem promessa de cura ou tratamento.</t>
         </is>
       </c>
     </row>
@@ -714,7 +761,7 @@
     <col width="44" customWidth="1" min="16" max="16"/>
     <col width="44" customWidth="1" min="17" max="17"/>
     <col width="44" customWidth="1" min="18" max="18"/>
-    <col width="50" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
     <col width="28" customWidth="1" min="20" max="22"/>
     <col width="24" customWidth="1" min="23" max="23"/>
     <col width="42" customWidth="1" min="24" max="24"/>
@@ -847,7 +894,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="140" customHeight="1">
+    <row r="2" ht="150" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>SKU</t>
@@ -945,7 +992,9 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Descrição comercial do produto (texto da marca)</t>
+          <t>Descrição comercial do produto
+TEXTO CORRIDO de 3 a 5 frases. NÃO repetir o nome do produto.
+Explique: para quem é, o que tem de especial, como ajuda o animal e como usar.</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">

</xml_diff>